<commit_message>
Log Fri posts, Thu IG URLs, calendar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwvMu8sUQkTnoofcUnh86
</commit_message>
<xml_diff>
--- a/ig-news/plan/hotcoin-content-calendar.xlsx
+++ b/ig-news/plan/hotcoin-content-calendar.xlsx
@@ -767,12 +767,12 @@
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>Live pick. Ready angle: Amazon + Strategy results</t>
+          <t>Suspected $5.5B Binance hack (scheduled; developing story, re-check at 15:40)</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>Myth vs Fact: "Sell in May, buy at Halloween". Tested on 30 years of S&amp;P data</t>
+          <t>Myth vs Fact: "Sell in May" would have halved your gains (scheduled)</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">

</xml_diff>

<commit_message>
Log Sat posts, Fri IG URLs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwvMu8sUQkTnoofcUnh86
</commit_message>
<xml_diff>
--- a/ig-news/plan/hotcoin-content-calendar.xlsx
+++ b/ig-news/plan/hotcoin-content-calendar.xlsx
@@ -807,12 +807,12 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Live pick. Fallback: Bitcoin whitepaper, 18 years (Oct 31, 2008)</t>
+          <t>Binance hack update: $6.3B, investigators point to North Korea (scheduled, Teng face cover)</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>Crypto 101: the 9-page whitepaper that started Bitcoin (timeline)</t>
+          <t>Crypto 101 ON THIS DAY: whitepaper turns 18, 9 pages -&gt; $1.5T (scheduled)</t>
         </is>
       </c>
       <c r="G8" s="26" t="inlineStr">

</xml_diff>